<commit_message>
Auto: 2026-09-30 scrape results
</commit_message>
<xml_diff>
--- a/results/auto_Cape_Town_Community_Development.xlsx
+++ b/results/auto_Cape_Town_Community_Development.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="44">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -533,9 +533,6 @@
       <c r="D3" t="s">
         <v>27</v>
       </c>
-      <c r="G3" t="s">
-        <v>43</v>
-      </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
@@ -584,9 +581,6 @@
       <c r="D6" t="s">
         <v>30</v>
       </c>
-      <c r="G6" t="s">
-        <v>43</v>
-      </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
@@ -601,9 +595,6 @@
       <c r="D7" t="s">
         <v>31</v>
       </c>
-      <c r="G7" t="s">
-        <v>43</v>
-      </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
@@ -618,9 +609,6 @@
       <c r="D8" t="s">
         <v>32</v>
       </c>
-      <c r="G8" t="s">
-        <v>43</v>
-      </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
@@ -635,9 +623,6 @@
       <c r="D9" t="s">
         <v>33</v>
       </c>
-      <c r="G9" t="s">
-        <v>43</v>
-      </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
@@ -652,9 +637,6 @@
       <c r="D10" t="s">
         <v>34</v>
       </c>
-      <c r="G10" t="s">
-        <v>43</v>
-      </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
@@ -668,9 +650,6 @@
       </c>
       <c r="D11" t="s">
         <v>35</v>
-      </c>
-      <c r="G11" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:7">

</xml_diff>